<commit_message>
PTCS 6 tracker: log Aug 17-20 results (day 18 of 35)
Dashboard DATA + tracker workbook updated with four more scoring days
(Gold 19 and Silver 15 spikes, Diamond 10 on Aug 20); elapsedDays 14 -> 18.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LvuavcVRWL5Y47m8wmR5G2
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -1903,64 +1903,192 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr"/>
-      <c r="B19" s="8" t="inlineStr"/>
-      <c r="C19" s="8" t="inlineStr"/>
-      <c r="D19" s="8" t="inlineStr"/>
-      <c r="E19" s="8" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr"/>
-      <c r="G19" s="8" t="inlineStr"/>
-      <c r="H19" s="8" t="inlineStr"/>
-      <c r="I19" s="8" t="inlineStr"/>
-      <c r="J19" s="8" t="inlineStr"/>
-      <c r="K19" s="8" t="inlineStr"/>
-      <c r="L19" s="8" t="inlineStr"/>
-      <c r="M19" s="8" t="inlineStr"/>
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Mon Aug 17</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>LOW BRONZE 2nd PLACE (64) +15 BRONZE. Return of the Bronze 17-32 (128) +3B; Bronze The Sequel 33-64 (128) +1B; Laptophound 5L Deadball 17-32 (128) +3 PDD; Struggling to Sleep DBL 9-16 (64) +3 PDD; OOTP and Chill 17-32 (64) +1 PDD; Diamond &amp; Friends Slots 17-32 (64) +1D/+1C. ZEROS: Monday Gold Floor Cap 65-128 (128, Op+Cp), Monday Wonky Historical Slots 65-128 (128, Gld+Cp), Late Silver 65-128 (128), Just Order Pizza D&amp;G 33-64 (64), Doc Rock Derby 33-64 (64), Trying to Look Busy D&amp;G 33-64 (64), Early Gold 65-128 (128)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr"/>
-      <c r="B20" s="8" t="inlineStr"/>
-      <c r="C20" s="8" t="inlineStr"/>
-      <c r="D20" s="8" t="inlineStr"/>
-      <c r="E20" s="8" t="inlineStr"/>
-      <c r="F20" s="8" t="inlineStr"/>
-      <c r="G20" s="8" t="inlineStr"/>
-      <c r="H20" s="8" t="inlineStr"/>
-      <c r="I20" s="8" t="inlineStr"/>
-      <c r="J20" s="8" t="inlineStr"/>
-      <c r="K20" s="8" t="inlineStr"/>
-      <c r="L20" s="8" t="inlineStr"/>
-      <c r="M20" s="8" t="inlineStr"/>
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Tue Aug 18</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="11" t="inlineStr">
+        <is>
+          <t>THIS COULD VE BEEN AN EMAIL RCK WINNER (64) +25 PD DAILY - 3rd win of the period. Late Silver 3rd/4th (128) +15 SILVER - best Silver result of the period. Bronze The Sequel 17-32 (128) +3B; Nocturnal Mixed Bag 5-8 (32) +3 PDD; Low Bronze 17-32 (64) +1B; Diamond Slots 17-32 (64) +1D/+1C. ZEROS: Mixed Up My Lunch 17-32 (32 - pays 0 there), Just Order Pizza D&amp;G 33-64 (64), Low Gold Retrospecticus 33-64 (64), Early Gold 65-128 (128), Laptophound 5L Deadball 65-128 (128), Bagels and Schmear 33-64 (64), Struggling to Sleep DBL 33-64 (64) | LATE ADD: Tuesday Sporer's Sandlot 33-64 (128, Gld+Cp+TW) +1G/+1C. (Nocturnal Mixed Bag re-appeared in a later screenshot - same event id 2550147, already counted, not double-logged.)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr"/>
-      <c r="B21" s="8" t="inlineStr"/>
-      <c r="C21" s="8" t="inlineStr"/>
-      <c r="D21" s="8" t="inlineStr"/>
-      <c r="E21" s="8" t="inlineStr"/>
-      <c r="F21" s="8" t="inlineStr"/>
-      <c r="G21" s="8" t="inlineStr"/>
-      <c r="H21" s="8" t="inlineStr"/>
-      <c r="I21" s="8" t="inlineStr"/>
-      <c r="J21" s="8" t="inlineStr"/>
-      <c r="K21" s="8" t="inlineStr"/>
-      <c r="L21" s="8" t="inlineStr"/>
-      <c r="M21" s="8" t="inlineStr"/>
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Wed Aug 19</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="11" t="inlineStr">
+        <is>
+          <t>QUIET DAY - 6 pts, mostly 33-64s. Late Silver 17-32 (128) +3S; Open Slots 17-32 (64) +1 OPEN/+1C; Laptophound 5L Deadball 33-64 (128) +1 PDD. ZEROS: Low Bronze 33-64 (64), Golden Heart 33-64 (64), Just Order Pizza D&amp;G 33-64 (64), Pitchers First 33-64 (64), Early Gold 65-128 (128), Bronze The Sequel 65-128 (128). Wednesday Ice to See You (Dia,TW, 256) ELIMINATED - placement unknown, unscored</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr"/>
-      <c r="B22" s="8" t="inlineStr"/>
-      <c r="C22" s="8" t="inlineStr"/>
-      <c r="D22" s="8" t="inlineStr"/>
-      <c r="E22" s="8" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr"/>
-      <c r="G22" s="8" t="inlineStr"/>
-      <c r="H22" s="8" t="inlineStr"/>
-      <c r="I22" s="8" t="inlineStr"/>
-      <c r="J22" s="8" t="inlineStr"/>
-      <c r="K22" s="8" t="inlineStr"/>
-      <c r="L22" s="8" t="inlineStr"/>
-      <c r="M22" s="8" t="inlineStr"/>
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Thu Aug 20</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="11" t="inlineStr">
+        <is>
+          <t>CWHIT CAP CHALLENGE 4 QUARTERFINAL (128, Gld+Cp) +10 GOLD/+10 CAP - biggest Cap day since Aug 3. Diamond Slots 9-16 (64) +3D/+3C; Thursday Silver Spectacular 65-128 (256) +1S; Return of the Bronze 33-64 (128) +1B. ZEROS: Goldfather II 33-64 (64), Trying to Look Busy D&amp;G 33-64 (64), Bronze The Sequel 65-128 (128). Thursday Overnight Under the Covers (PD Weekly, 256) ELIMINATED - 3rd time this period, unscored</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
Log Aug 25-26 results: +28 (796 total, day 24)
Aug 25 +13 (Diamond Slots + Low Diamond 9-16s), Aug 26 +15 (5L Deadball
5th-8th = +10 PDD, best PD finish of the period). PD Weekly: Adrenaline
Rush and Ice to See You both eliminated - PDW stays 41. Diamond now 114,
13 past its estimated target.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LvuavcVRWL5Y47m8wmR5G2
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="178">
   <si>
     <t xml:space="preserve">PTCS 6 — All 10 Categories (Aug 3 – Sep 6)</t>
   </si>
@@ -364,6 +364,18 @@
   </si>
   <si>
     <t xml:space="preserve">LOW DIAMOND 3rd/4th (64) +10 DIAMOND - Diamond crosses the 101-pt estimated target. Wonky Historical Slots 17-32 (128, Gld+Cp+TW) +3G/+3C; Just Order Pizza D&amp;G 9-16 (64) +3 PDD; Gold Slots 17-32 (64) +1G/+1C; Up And At Them Bronze 65-128 (256) +1B. Monday Getting it Started (PD Weekly, 256) ELIMINATED - unscored. ZEROS: Tuck in Time + Snack Time 17-32 (32s pay 0), Silver Slots, Silver Heart, Hitters First, Open Slots 33-64 (64), Gold Floor Cap, 6L Power Play, Bronze OOTP Era, 5L Deadball 65-128 (128).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tue Aug 25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIAMOND SLOTS 9-16 (64) +3D/+3C; Low Diamond 9-16 (64) +3D; PDD singles: 6L Power Play 33-64 (128), Just Order Pizza 17-32 (64), Trying to Look Busy 17-32 (64), 5L Deadball 33-64 (128). Tuesday Evening Adrenaline Rush (PD WEEKLY, 256) ELIMINATED - 0. ZEROS: Sporer's Sandlot 65-128 + Up to 1969 33-64 (TW), Late Silver + Early Gold 65-128 (128), Gold Slots 33-64 (64), This Could've Been an Email 33-64 (64).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wed Aug 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5L DEADBALL 5th-8th (128) +10 PDD - best PD Daily finish of the period. PDD singles: 6L Power Play 33-64 (128), Good Orderly Evening 17-32 (64). Diamond &amp; Friends Slots 17-32 (64) +1D/+1C; Late Silver 33-64 (128) +1S. Wednesday Ice to See You (256, Dia weekly) ELIMINATED. ZEROS: Bronze Only Cap, Bronze 1910-59, Gold Slots, Trying to Look Busy, Doc Rock Derby 33-64 (64s); Early Gold + Night of the Living Deadball 65-128 (128); Up Late with Rich 17-32 (32 pays 0). W-1950-to-Now excluded.</t>
   </si>
   <si>
     <t xml:space="preserve">The Championship Ladder — PTCS → PTMS → PTWC</t>
@@ -1120,18 +1132,18 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUM('Daily Log'!E5:E52)</f>
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>129</v>
       </c>
       <c r="D7" s="7" t="n">
         <f aca="false">MAX(0,C7-B7)</f>
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">ROUND(D7/5,1)</f>
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">ROUND(D7/35,1)</f>
@@ -1142,7 +1154,7 @@
       </c>
       <c r="H7" s="9" t="str">
         <f aca="false">IF(B7&gt;=C7,"QUALIFIED","+"&amp;TEXT(D7,"0")&amp;" to go")</f>
-        <v>+43 to go</v>
+        <v>+42 to go</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1182,7 +1194,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM('Daily Log'!G5:G52)</f>
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>101</v>
@@ -1275,29 +1287,29 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">SUM('Daily Log'!J5:J52)</f>
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>179</v>
       </c>
       <c r="D12" s="7" t="n">
         <f aca="false">MAX(0,C12-B12)</f>
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">ROUND(D12/5,1)</f>
-        <v>13.8</v>
+        <v>13</v>
       </c>
       <c r="F12" s="7" t="n">
         <f aca="false">ROUND(D12/35,1)</f>
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>24</v>
       </c>
       <c r="H12" s="9" t="str">
         <f aca="false">IF(B12&gt;=C12,"QUALIFIED","+"&amp;TEXT(D12,"0")&amp;" to go")</f>
-        <v>+69 to go</v>
+        <v>+65 to go</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1306,29 +1318,29 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">SUM('Daily Log'!K5:K52)</f>
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>334</v>
       </c>
       <c r="D13" s="7" t="n">
         <f aca="false">MAX(0,C13-B13)</f>
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">ROUND(D13/5,1)</f>
-        <v>24.4</v>
+        <v>21.2</v>
       </c>
       <c r="F13" s="7" t="n">
         <f aca="false">ROUND(D13/35,1)</f>
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>26</v>
       </c>
       <c r="H13" s="9" t="str">
         <f aca="false">IF(B13&gt;=C13,"QUALIFIED","+"&amp;TEXT(D13,"0")&amp;" to go")</f>
-        <v>+122 to go</v>
+        <v>+106 to go</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2507,34 +2519,86 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
-      <c r="L27" s="9"/>
-      <c r="M27" s="9"/>
+      <c r="A27" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="12" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
-      <c r="M28" s="9"/>
+      <c r="A28" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="L28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="12" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="9"/>
@@ -2925,151 +2989,151 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>300</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>40</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>20</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="5" t="n">
@@ -3080,7 +3144,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>2</v>
@@ -3088,7 +3152,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>1</v>
@@ -3096,21 +3160,21 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>3</v>
@@ -3121,10 +3185,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C18" s="7" t="n">
         <v>0</v>
@@ -3136,15 +3200,15 @@
         <v>0</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C19" s="7" t="n">
         <v>0</v>
@@ -3156,15 +3220,15 @@
         <v>0</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C20" s="7" t="n">
         <v>1</v>
@@ -3176,15 +3240,15 @@
         <v>1</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>20</v>
@@ -3196,15 +3260,15 @@
         <v>20</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C22" s="7" t="n">
         <v>9</v>
@@ -3216,12 +3280,12 @@
         <v>14</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7" t="n">
@@ -3237,52 +3301,52 @@
         <v>35</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3290,17 +3354,17 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3308,17 +3372,17 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3326,7 +3390,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ingest diamond/weekly/PD batch; log Aug 27-28 (+43, 839 total)
Archive now 291 files / 43 series / 25,021 observed rows — the two
Laptophound PD series arrive as the biggest in the archive (1,555 +
1,324 cards). Catalog: Laptop*/Doc Rock names now flag isDraft (the
databotai rows carried no PD marker) and 5ldeadball/6lpowerplay pin to
their real rows; draft series are excluded from the projection fit
(r2 recovered .309 -> .345/.322, best pitcher fit yet). Results: Thu
+33 (Silver Slots 3rd/4th = +10 Silver/+10 Cap, first PDW point since
Aug 22), Fri +10 so far (Diamond Heart 5th-8th). No overlap with the
Aug 26 log — screenshot's Aug 26 rows were already recorded.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LvuavcVRWL5Y47m8wmR5G2
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="182">
   <si>
     <t xml:space="preserve">PTCS 6 — All 10 Categories (Aug 3 – Sep 6)</t>
   </si>
@@ -376,6 +376,18 @@
   </si>
   <si>
     <t xml:space="preserve">5L DEADBALL 5th-8th (128) +10 PDD - best PD Daily finish of the period. PDD singles: 6L Power Play 33-64 (128), Good Orderly Evening 17-32 (64). Diamond &amp; Friends Slots 17-32 (64) +1D/+1C; Late Silver 33-64 (128) +1S. Wednesday Ice to See You (256, Dia weekly) ELIMINATED. ZEROS: Bronze Only Cap, Bronze 1910-59, Gold Slots, Trying to Look Busy, Doc Rock Derby 33-64 (64s); Early Gold + Night of the Living Deadball 65-128 (128); Up Late with Rich 17-32 (32 pays 0). W-1950-to-Now excluded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thu Aug 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SILVER SLOTS 3rd/4th (64) +10 SILVER/+10 CAP - biggest Silver+Cap hit of the period. Just Order Pizza 5-8 (64) +6 PDD; CWhit Cap Challenge 4 33-64 (128) +1G/+1C; PDD singles: 6L Power Play (167), Pitchers First 17-32 (64), 5L Deadball (166); Bronze 1910-59 17-32 (64) +1B; Thursday Overnight Under the Covers 65-128 (256) +1 PDW - first PDW point since Aug 22. Weeklies ELIMINATED: Gold Rush, Silver Spectacular. ZEROS: Golden Childhood, Bronze Only Cap 167, Late Silver, Diamond Slots 167, Bronze OOTP Era, Could've Been an Email 166, Double Espresso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fri Aug 28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diamond Heart 5-8 (64) +6 DIAMOND. Snack Time on the Ladder 5-8 (32) +3 PDD; 5L Deadball 33-64 (128) +1 PDD. Friday Draft About Nothing (PDW, 256) ELIMINATED. ZEROS: Open Slots, Early Gold 167, Gold Slots 167. Partial day - morning screenshot, expect late adds.</t>
   </si>
   <si>
     <t xml:space="preserve">The Championship Ladder — PTCS → PTMS → PTWC</t>
@@ -1101,18 +1113,18 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">SUM('Daily Log'!D5:D52)</f>
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>130</v>
       </c>
       <c r="D6" s="7" t="n">
         <f aca="false">MAX(0,C6-B6)</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">ROUND(D6/5,1)</f>
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">ROUND(D6/35,1)</f>
@@ -1123,7 +1135,7 @@
       </c>
       <c r="H6" s="9" t="str">
         <f aca="false">IF(B6&gt;=C6,"QUALIFIED","+"&amp;TEXT(D6,"0")&amp;" to go")</f>
-        <v>+19 to go</v>
+        <v>+18 to go</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1132,29 +1144,29 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUM('Daily Log'!E5:E52)</f>
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>129</v>
       </c>
       <c r="D7" s="7" t="n">
         <f aca="false">MAX(0,C7-B7)</f>
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">ROUND(D7/5,1)</f>
-        <v>8.4</v>
+        <v>6.4</v>
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">ROUND(D7/35,1)</f>
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="H7" s="9" t="str">
         <f aca="false">IF(B7&gt;=C7,"QUALIFIED","+"&amp;TEXT(D7,"0")&amp;" to go")</f>
-        <v>+42 to go</v>
+        <v>+32 to go</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1163,18 +1175,18 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">SUM('Daily Log'!F5:F52)</f>
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>114</v>
       </c>
       <c r="D8" s="7" t="n">
         <f aca="false">MAX(0,C8-B8)</f>
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E8" s="7" t="n">
         <f aca="false">ROUND(D8/5,1)</f>
-        <v>7.2</v>
+        <v>7</v>
       </c>
       <c r="F8" s="7" t="n">
         <f aca="false">ROUND(D8/35,1)</f>
@@ -1185,7 +1197,7 @@
       </c>
       <c r="H8" s="9" t="str">
         <f aca="false">IF(B8&gt;=C8,"QUALIFIED","+"&amp;TEXT(D8,"0")&amp;" to go")</f>
-        <v>+36 to go</v>
+        <v>+35 to go</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1194,7 +1206,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM('Daily Log'!G5:G52)</f>
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>101</v>
@@ -1287,29 +1299,29 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">SUM('Daily Log'!J5:J52)</f>
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>179</v>
       </c>
       <c r="D12" s="7" t="n">
         <f aca="false">MAX(0,C12-B12)</f>
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">ROUND(D12/5,1)</f>
-        <v>13</v>
+        <v>10.8</v>
       </c>
       <c r="F12" s="7" t="n">
         <f aca="false">ROUND(D12/35,1)</f>
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>24</v>
       </c>
       <c r="H12" s="9" t="str">
         <f aca="false">IF(B12&gt;=C12,"QUALIFIED","+"&amp;TEXT(D12,"0")&amp;" to go")</f>
-        <v>+65 to go</v>
+        <v>+54 to go</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1318,29 +1330,29 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">SUM('Daily Log'!K5:K52)</f>
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>334</v>
       </c>
       <c r="D13" s="7" t="n">
         <f aca="false">MAX(0,C13-B13)</f>
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">ROUND(D13/5,1)</f>
-        <v>21.2</v>
+        <v>18.6</v>
       </c>
       <c r="F13" s="7" t="n">
         <f aca="false">ROUND(D13/35,1)</f>
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>26</v>
       </c>
       <c r="H13" s="9" t="str">
         <f aca="false">IF(B13&gt;=C13,"QUALIFIED","+"&amp;TEXT(D13,"0")&amp;" to go")</f>
-        <v>+106 to go</v>
+        <v>+93 to go</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1349,29 +1361,29 @@
       </c>
       <c r="B14" s="6" t="n">
         <f aca="false">SUM('Daily Log'!L5:L52)</f>
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C14" s="7" t="n">
         <v>96</v>
       </c>
       <c r="D14" s="7" t="n">
         <f aca="false">MAX(0,C14-B14)</f>
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E14" s="7" t="n">
         <f aca="false">ROUND(D14/5,1)</f>
-        <v>11</v>
+        <v>10.8</v>
       </c>
       <c r="F14" s="7" t="n">
         <f aca="false">ROUND(D14/35,1)</f>
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>28</v>
       </c>
       <c r="H14" s="9" t="str">
         <f aca="false">IF(B14&gt;=C14,"QUALIFIED","+"&amp;TEXT(D14,"0")&amp;" to go")</f>
-        <v>+55 to go</v>
+        <v>+54 to go</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2601,34 +2613,86 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9"/>
-      <c r="K29" s="9"/>
-      <c r="L29" s="9"/>
-      <c r="M29" s="9"/>
+      <c r="A29" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" s="12" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="9"/>
-      <c r="K30" s="9"/>
-      <c r="L30" s="9"/>
-      <c r="M30" s="9"/>
+      <c r="A30" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="12" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="9"/>
@@ -2989,151 +3053,151 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>300</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>40</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>20</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="5" t="n">
@@ -3144,7 +3208,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>2</v>
@@ -3152,7 +3216,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>1</v>
@@ -3160,21 +3224,21 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>3</v>
@@ -3185,10 +3249,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C18" s="7" t="n">
         <v>0</v>
@@ -3200,15 +3264,15 @@
         <v>0</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C19" s="7" t="n">
         <v>0</v>
@@ -3220,15 +3284,15 @@
         <v>0</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C20" s="7" t="n">
         <v>1</v>
@@ -3240,15 +3304,15 @@
         <v>1</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>20</v>
@@ -3260,15 +3324,15 @@
         <v>20</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C22" s="7" t="n">
         <v>9</v>
@@ -3280,12 +3344,12 @@
         <v>14</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7" t="n">
@@ -3301,52 +3365,52 @@
         <v>35</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3354,17 +3418,17 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3372,17 +3436,17 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3390,7 +3454,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Log Aug 28-29: Friday re-scored to +78 - best day of PTCS 6
Golden Heart WINNER (+25 Gold, first W of the period), Silver Slots
2nd (+15 Silver/+15 Cap), Silver Heart 3rd/4th (+10 S), on top of the
morning's Diamond Heart 5-8. Friday: 10 -> 78. Saturday opens +3.
Total 910 at day 27; Silver 122, Gold 104, Cap 140, Diamond 120.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LvuavcVRWL5Y47m8wmR5G2
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="184">
   <si>
     <t xml:space="preserve">PTCS 6 — All 10 Categories (Aug 3 – Sep 6)</t>
   </si>
@@ -387,7 +387,13 @@
     <t xml:space="preserve">Fri Aug 28</t>
   </si>
   <si>
-    <t xml:space="preserve">Diamond Heart 5-8 (64) +6 DIAMOND. Snack Time on the Ladder 5-8 (32) +3 PDD; 5L Deadball 33-64 (128) +1 PDD. Friday Draft About Nothing (PDW, 256) ELIMINATED. ZEROS: Open Slots, Early Gold 167, Gold Slots 167. Partial day - morning screenshot, expect late adds.</t>
+    <t xml:space="preserve">BEST DAY OF THE PERIOD (+78). GOLDEN HEART WINNER (64) +25 GOLD - first tournament WIN of PTCS 6. Silver Slots 2ND (64) +15 SILVER/+15 CAP; Silver Heart 3rd/4th (64) +10 SILVER; Diamond Heart 5-8 (64) +6 D; Doc Rock Derby 9-16 (64) +3 PDD; Snack Time 5-8 (32) +3 PDD; 5L Deadball 33-64 (128) +1 PDD. Draft About Nothing (PDW) eliminated. ZEROS: Open Slots, Early Gold, Gold Slots, 6L Power Play 168, Late Silver 168, Silver Slamboree. LATE ADDS from Aug 29 screenshot amended this day (+68 over the morning partial).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sat Aug 29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Struggling to Sleep 9-16 (64) +3 PDD. Partial day - morning screenshot.</t>
   </si>
   <si>
     <t xml:space="preserve">The Championship Ladder — PTCS → PTMS → PTWC</t>
@@ -1144,29 +1150,29 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUM('Daily Log'!E5:E52)</f>
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>129</v>
       </c>
       <c r="D7" s="7" t="n">
         <f aca="false">MAX(0,C7-B7)</f>
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">ROUND(D7/5,1)</f>
-        <v>6.4</v>
+        <v>1.4</v>
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">ROUND(D7/35,1)</f>
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>14</v>
       </c>
       <c r="H7" s="9" t="str">
         <f aca="false">IF(B7&gt;=C7,"QUALIFIED","+"&amp;TEXT(D7,"0")&amp;" to go")</f>
-        <v>+32 to go</v>
+        <v>+7 to go</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1175,29 +1181,29 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">SUM('Daily Log'!F5:F52)</f>
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>114</v>
       </c>
       <c r="D8" s="7" t="n">
         <f aca="false">MAX(0,C8-B8)</f>
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="E8" s="7" t="n">
         <f aca="false">ROUND(D8/5,1)</f>
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F8" s="7" t="n">
         <f aca="false">ROUND(D8/35,1)</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>16</v>
       </c>
       <c r="H8" s="9" t="str">
         <f aca="false">IF(B8&gt;=C8,"QUALIFIED","+"&amp;TEXT(D8,"0")&amp;" to go")</f>
-        <v>+35 to go</v>
+        <v>+10 to go</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1299,29 +1305,29 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">SUM('Daily Log'!J5:J52)</f>
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>179</v>
       </c>
       <c r="D12" s="7" t="n">
         <f aca="false">MAX(0,C12-B12)</f>
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">ROUND(D12/5,1)</f>
-        <v>10.8</v>
+        <v>7.8</v>
       </c>
       <c r="F12" s="7" t="n">
         <f aca="false">ROUND(D12/35,1)</f>
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>24</v>
       </c>
       <c r="H12" s="9" t="str">
         <f aca="false">IF(B12&gt;=C12,"QUALIFIED","+"&amp;TEXT(D12,"0")&amp;" to go")</f>
-        <v>+54 to go</v>
+        <v>+39 to go</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1330,29 +1336,29 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">SUM('Daily Log'!K5:K52)</f>
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>334</v>
       </c>
       <c r="D13" s="7" t="n">
         <f aca="false">MAX(0,C13-B13)</f>
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">ROUND(D13/5,1)</f>
-        <v>18.6</v>
+        <v>17.4</v>
       </c>
       <c r="F13" s="7" t="n">
         <f aca="false">ROUND(D13/35,1)</f>
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>26</v>
       </c>
       <c r="H13" s="9" t="str">
         <f aca="false">IF(B13&gt;=C13,"QUALIFIED","+"&amp;TEXT(D13,"0")&amp;" to go")</f>
-        <v>+93 to go</v>
+        <v>+87 to go</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2667,10 +2673,10 @@
         <v>0</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>6</v>
@@ -2682,10 +2688,10 @@
         <v>0</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L30" s="7" t="n">
         <v>0</v>
@@ -2695,19 +2701,45 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
+      <c r="A31" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="12" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="9"/>
@@ -3053,151 +3085,151 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="F5" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>300</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>40</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>20</v>
       </c>
       <c r="D10" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>142</v>
-      </c>
       <c r="F10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="5" t="n">
@@ -3208,7 +3240,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>2</v>
@@ -3216,7 +3248,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>1</v>
@@ -3224,21 +3256,21 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>3</v>
@@ -3249,10 +3281,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C18" s="7" t="n">
         <v>0</v>
@@ -3264,35 +3296,35 @@
         <v>0</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="12" t="s">
         <v>154</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C20" s="7" t="n">
         <v>1</v>
@@ -3304,15 +3336,15 @@
         <v>1</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>20</v>
@@ -3324,15 +3356,15 @@
         <v>20</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C22" s="7" t="n">
         <v>9</v>
@@ -3344,12 +3376,12 @@
         <v>14</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7" t="n">
@@ -3365,52 +3397,52 @@
         <v>35</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3418,17 +3450,17 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3436,17 +3468,17 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3454,7 +3486,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PTCS6: complete day 28 (Aug 30) from full list — +10, total 1001
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -2511,7 +2511,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="20" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>6</v>
@@ -2520,23 +2520,23 @@
         <v>0</v>
       </c>
       <c r="H32" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" s="20" t="n">
         <v>0</v>
       </c>
       <c r="J32" s="20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K32" s="20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L32" s="20" t="n">
         <v>0</v>
       </c>
       <c r="M32" s="25" t="inlineStr">
         <is>
-          <t>Gold+Cap doubles: Sunday High Iron Floor and Gold Ceiling 17-32 (128, Gld+Cp+TW) +3 G/+3 C; Gold Slots 9-16 (64) +3 G/+3 C. PDD: Struggling to Sleep 9-16 (64) +3, 5L Deadball 33-64 (128) +1. ZEROS: Low Gold Retrospecticus 33-64 (64), Bagels and Schmear 33-64 (64). Partial day - evening screenshot.</t>
+          <t>Gold+Cap doubles: Sunday High Iron Floor and Gold Ceiling 17-32 (128, Gld+Cp+TW) +3 G/+3 C; Gold Slots 9-16 (64) +3 G/+3 C. PDD: Struggling to Sleep 9-16 (64) +3, 5L Deadball 33-64 (128) +1. ZEROS: Low Gold Retrospecticus 33-64 (64), Bagels and Schmear 33-64 (64). LATE ADDS from the Sep 1 full-list screenshots (+10): Silver Heart 5-8 (64) +6 S; Late Silver 33-64 (128) +1 S; Sunday Open Slots 33-64 (128, Op+Cp+TW) +1 O/+1 C; Rocking Chair Lunch 17-32 (64) +1 PDD. LATE ZEROS: Silver Slots 33-64 (64); 6L Power Play 65-128 (128); Bronze OOTP Era 65-128 (128); Sunday Up and Down the Ladder 65-128 (128, PD WEEKLY). Day now complete.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PTCS6 day 30 (Tue Sep 1): +40, running total 1041
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDzMYYjBuFssTrjcZrtJCL
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -2588,19 +2588,51 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="14">
-      <c r="A34" s="22" t="n"/>
-      <c r="B34" s="22" t="n"/>
-      <c r="C34" s="22" t="n"/>
-      <c r="D34" s="22" t="n"/>
-      <c r="E34" s="22" t="n"/>
-      <c r="F34" s="22" t="n"/>
-      <c r="G34" s="22" t="n"/>
-      <c r="H34" s="22" t="n"/>
-      <c r="I34" s="22" t="n"/>
-      <c r="J34" s="22" t="n"/>
-      <c r="K34" s="22" t="n"/>
-      <c r="L34" s="22" t="n"/>
-      <c r="M34" s="22" t="n"/>
+      <c r="A34" s="25" t="inlineStr">
+        <is>
+          <t>Tue Sep 1</t>
+        </is>
+      </c>
+      <c r="B34" s="25" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="K34" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="L34" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="25" t="inlineStr">
+        <is>
+          <t>BRONZE PTCS 3 REPLAY SLOTS 3rd/4th (64) +10 B/+10 CAP - biggest Bronze hit of the period and the swing that puts Bronze within 4 of target. 6L Power Play 5-8 (128) +10 PDD - best PD Daily result since the Aug 26 Deadball 5-8. Perfecto Primetime 9-16 (64) +3 PDD; Early Gold 17-32 (128) +3 G; Silver Slots 17-32 (64) +1 S/+1 C; Diamond &amp; Friends Slots 17-32 (64) +1 D/+1 C. ZEROS: Perfectly Silver 33-64 (64); All-Gold 33-64 (64); All-Silver 33-64 (64); Bronze OOTP Era 65-128 (128); 5L Deadball 65-128 (128); Tuesday Up to 1969 65-128 (128, Op+TW).</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="14">
       <c r="A35" s="22" t="n"/>

</xml_diff>

<commit_message>
PTCS6: swap estimated targets for real 128th-place berth lines from the dumps
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDzMYYjBuFssTrjcZrtJCL
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -501,7 +501,7 @@
     <row r="2" ht="15" customHeight="1" s="14">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>5-week period. Targets = PTCS5 cutoff × 5/4 (estimates — replace with official once week-1 standings post).</t>
+          <t>5-week period. Targets = real 128th-place berth lines from the Aug 24/31 community dumps, projected to Sep 6. (Previously PTCS5 cutoff x 5/4, which ran high.)</t>
         </is>
       </c>
     </row>
@@ -518,7 +518,7 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>Target (est)</t>
+          <t>Target (128th line)</t>
         </is>
       </c>
       <c r="D4" s="17" t="inlineStr">
@@ -558,7 +558,7 @@
         <v/>
       </c>
       <c r="C5" s="20" t="n">
-        <v>135</v>
+        <v>107</v>
       </c>
       <c r="D5" s="20">
         <f>MAX(0,C5-B5)</f>
@@ -593,7 +593,7 @@
         <v/>
       </c>
       <c r="C6" s="20" t="n">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D6" s="20">
         <f>MAX(0,C6-B6)</f>
@@ -628,7 +628,7 @@
         <v/>
       </c>
       <c r="C7" s="20" t="n">
-        <v>129</v>
+        <v>105</v>
       </c>
       <c r="D7" s="20">
         <f>MAX(0,C7-B7)</f>
@@ -663,7 +663,7 @@
         <v/>
       </c>
       <c r="C8" s="20" t="n">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="D8" s="20">
         <f>MAX(0,C8-B8)</f>
@@ -698,7 +698,7 @@
         <v/>
       </c>
       <c r="C9" s="20" t="n">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="D9" s="20">
         <f>MAX(0,C9-B9)</f>
@@ -733,7 +733,7 @@
         <v/>
       </c>
       <c r="C10" s="20" t="n">
-        <v>129</v>
+        <v>53</v>
       </c>
       <c r="D10" s="20">
         <f>MAX(0,C10-B10)</f>
@@ -768,7 +768,7 @@
         <v/>
       </c>
       <c r="C11" s="20" t="n">
-        <v>176</v>
+        <v>125</v>
       </c>
       <c r="D11" s="20">
         <f>MAX(0,C11-B11)</f>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="C12" s="20" t="n">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="D12" s="20">
         <f>MAX(0,C12-B12)</f>
@@ -838,7 +838,7 @@
         <v/>
       </c>
       <c r="C13" s="20" t="n">
-        <v>334</v>
+        <v>315</v>
       </c>
       <c r="D13" s="20">
         <f>MAX(0,C13-B13)</f>
@@ -873,7 +873,7 @@
         <v/>
       </c>
       <c r="C14" s="20" t="n">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="D14" s="20">
         <f>MAX(0,C14-B14)</f>

</xml_diff>

<commit_message>
PTCS6 day 31 (Wed Sep 2, partial): +3 Open, total 1044
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDzMYYjBuFssTrjcZrtJCL
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -2635,19 +2635,51 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="14">
-      <c r="A35" s="22" t="n"/>
-      <c r="B35" s="22" t="n"/>
-      <c r="C35" s="22" t="n"/>
-      <c r="D35" s="22" t="n"/>
-      <c r="E35" s="22" t="n"/>
-      <c r="F35" s="22" t="n"/>
-      <c r="G35" s="22" t="n"/>
-      <c r="H35" s="22" t="n"/>
-      <c r="I35" s="22" t="n"/>
-      <c r="J35" s="22" t="n"/>
-      <c r="K35" s="22" t="n"/>
-      <c r="L35" s="22" t="n"/>
-      <c r="M35" s="22" t="n"/>
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>Wed Sep 2</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="25" t="inlineStr">
+        <is>
+          <t>Wednesday 1950 to Now 17-32 (128, Op+TW) +3 OPEN - counted per the game's own Op tag; note the dump model currently EXCLUDES this event, so it may not show up in the community Open standings. ZEROS: Open Slots 33-64 (64, Op+Cp); Early Gold 65-128 (128). Partial day - still playing.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="14">
       <c r="A36" s="22" t="n"/>

</xml_diff>

<commit_message>
Adopt CWhit's Projected QP as the PTCS6 targets
His current-128 column measures the same Aug 31 dump my model reads, which
grades the mapping: within ~6 on Cap and PD Daily, 4-13 low across the tier
categories, and 42-55 low on Live and Open - the categories where categoriesOf
drops qualifying events.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDzMYYjBuFssTrjcZrtJCL
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -501,7 +501,7 @@
     <row r="2" ht="15" customHeight="1" s="14">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>5-week period. Targets = real 128th-place berth lines from the Aug 24/31 community dumps, projected to Sep 6. (Previously PTCS5 cutoff x 5/4, which ran high.)</t>
+          <t>5-week period. Targets = CWhit's Projected QP (read 2026-09-02). His current-128 column is the live cutoff as of the Aug 31 dump.</t>
         </is>
       </c>
     </row>
@@ -518,7 +518,7 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>Target (128th line)</t>
+          <t>Target (CWhit proj)</t>
         </is>
       </c>
       <c r="D4" s="17" t="inlineStr">
@@ -558,7 +558,7 @@
         <v/>
       </c>
       <c r="C5" s="20" t="n">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="D5" s="20">
         <f>MAX(0,C5-B5)</f>
@@ -593,7 +593,7 @@
         <v/>
       </c>
       <c r="C6" s="20" t="n">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="D6" s="20">
         <f>MAX(0,C6-B6)</f>
@@ -628,7 +628,7 @@
         <v/>
       </c>
       <c r="C7" s="20" t="n">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="D7" s="20">
         <f>MAX(0,C7-B7)</f>
@@ -663,7 +663,7 @@
         <v/>
       </c>
       <c r="C8" s="20" t="n">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="D8" s="20">
         <f>MAX(0,C8-B8)</f>
@@ -698,7 +698,7 @@
         <v/>
       </c>
       <c r="C9" s="20" t="n">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="D9" s="20">
         <f>MAX(0,C9-B9)</f>
@@ -733,7 +733,7 @@
         <v/>
       </c>
       <c r="C10" s="20" t="n">
-        <v>53</v>
+        <v>120</v>
       </c>
       <c r="D10" s="20">
         <f>MAX(0,C10-B10)</f>
@@ -768,7 +768,7 @@
         <v/>
       </c>
       <c r="C11" s="20" t="n">
-        <v>125</v>
+        <v>175</v>
       </c>
       <c r="D11" s="20">
         <f>MAX(0,C11-B11)</f>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="C12" s="20" t="n">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D12" s="20">
         <f>MAX(0,C12-B12)</f>
@@ -838,7 +838,7 @@
         <v/>
       </c>
       <c r="C13" s="20" t="n">
-        <v>315</v>
+        <v>347</v>
       </c>
       <c r="D13" s="20">
         <f>MAX(0,C13-B13)</f>
@@ -873,7 +873,7 @@
         <v/>
       </c>
       <c r="C14" s="20" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="D14" s="20">
         <f>MAX(0,C14-B14)</f>

</xml_diff>

<commit_message>
PTCS6: log Fri Sep 4 (+31) — Bronze 1910-59 WINNER, Bronze qualifies
Bronze 1910-59 1st (64) +25 Bronze carries the category to 152/133, the
fifth qualified alongside Silver, Gold, Diamond and Cap. Low Diamond 9-16
+3 D; All-Silver 9-16 +3 PDD; 5L Deadball 65-128 = 0.

Period total 1,142 through day 33. Partial day — logged at 6pm Central.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RG3WVSzFi65E25C24N7im4
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="196">
   <si>
     <t xml:space="preserve">PTCS 6 — All 10 Categories (Aug 3 – Sep 6)</t>
   </si>
@@ -424,6 +424,12 @@
   </si>
   <si>
     <t xml:space="preserve">CWHIT'S CAP CHALLENGE 4 3rd/4th (128, Gld+Cp+TW) +15 GOLD/+15 CAP - best Cap result of the period and the biggest Gold hit since the Aug 28 Golden Heart win. Thursday Silver Spectacular 9-16 (256, Slv+TW) +10 SILVER - TW carries no standing, Silver only. Silver &amp; Friends Slots 9-16 (64) +3 S/+3 C; Silver Only Cap 17-32 (64) +1 S/+1 C; Silver Slots 17-32 (64) +1 S/+1 C. PDD: Perfecto Primetime 9-16 (64) +3, All-Gold 9-16 (64) +3, Perfecto Morning 9-16 (64) +3, High Heat in the Morning 17-32 (64) +1, Struggling to Sleep - DBL 17-32 (64) +1. ZEROS: Bronze PTCS 3 Replay Slots 33-64 (64); Low Silver Only 33-64 (64); Low Diamond 33-64 (64); Bronze 1910-59 33-64 (64); 6L Power Play 65-128 (128); 5L Deadball 65-128 (128). ELIMINATED/unscored: Thursday Night Gold Rush (256, Gld+TW); Thursday Overnight Under the Covers (256, PD WEEKLY). Screenshot showed no Sep 4 group, so Sep 3 may still take late adds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fri Sep 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRONZE 1910-59 WINNER (64) +25 BRONZE - first win since the Aug 28 Golden Heart, and it carries Bronze past target (152/133). Low Diamond 9-16 (64) +3 D; All-Silver 9-16 (64) +3 PDD. ZERO: 5L Deadball 65-128 (128). Partial day - four events resolved as of 6pm Central, all run numbers exactly +1 on their Sep 3 counterparts.</t>
   </si>
   <si>
     <t xml:space="preserve">The Championship Ladder — PTCS → PTMS → PTWC</t>
@@ -1149,29 +1155,29 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">SUM('Daily Log'!D5:D52)</f>
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>133</v>
       </c>
       <c r="D6" s="7" t="n">
         <f aca="false">MAX(0,C6-B6)</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">ROUND(D6/5,1)</f>
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">ROUND(D6/35,1)</f>
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="9" t="str">
         <f aca="false">IF(B6&gt;=C6,"QUALIFIED","+"&amp;TEXT(D6,"0")&amp;" to go")</f>
-        <v>+6 to go</v>
+        <v>QUALIFIED</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1242,7 +1248,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM('Daily Log'!G5:G52)</f>
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>99</v>
@@ -1366,29 +1372,29 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">SUM('Daily Log'!K5:K52)</f>
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>347</v>
       </c>
       <c r="D13" s="7" t="n">
         <f aca="false">MAX(0,C13-B13)</f>
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">ROUND(D13/5,1)</f>
-        <v>10</v>
+        <v>9.4</v>
       </c>
       <c r="F13" s="7" t="n">
         <f aca="false">ROUND(D13/35,1)</f>
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>26</v>
       </c>
       <c r="H13" s="9" t="str">
         <f aca="false">IF(B13&gt;=C13,"QUALIFIED","+"&amp;TEXT(D13,"0")&amp;" to go")</f>
-        <v>+50 to go</v>
+        <v>+47 to go</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2977,19 +2983,45 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="9"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="9"/>
-      <c r="J37" s="9"/>
-      <c r="K37" s="9"/>
-      <c r="L37" s="9"/>
-      <c r="M37" s="9"/>
+      <c r="A37" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="12" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="9"/>
@@ -3245,151 +3277,151 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>138</v>
-      </c>
       <c r="F5" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>300</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>40</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>20</v>
       </c>
       <c r="D10" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>154</v>
-      </c>
       <c r="F10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="5" t="n">
@@ -3400,7 +3432,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>2</v>
@@ -3408,7 +3440,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>1</v>
@@ -3416,21 +3448,21 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>3</v>
@@ -3441,10 +3473,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C18" s="7" t="n">
         <v>0</v>
@@ -3456,35 +3488,35 @@
         <v>0</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="12" t="s">
         <v>166</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C20" s="7" t="n">
         <v>1</v>
@@ -3496,15 +3528,15 @@
         <v>1</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>20</v>
@@ -3516,15 +3548,15 @@
         <v>20</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C22" s="7" t="n">
         <v>9</v>
@@ -3536,12 +3568,12 @@
         <v>14</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7" t="n">
@@ -3557,52 +3589,52 @@
         <v>35</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3610,17 +3642,17 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3628,17 +3660,17 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3646,7 +3678,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PTCS6: amend Sep 4 to +51 — Silver Only Cap 3rd/4th
Daily Silver Only Cap 3rd/4th (64) +10 Silver/+10 Cap; Low Silver Only
33-64 (64) = 0. Day now 51: Bronze 25, Silver 10, Cap 10, Diamond 3, PDD 3.

Silver 164/119, Cap 196/161. Period total 1,162 through day 33.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RG3WVSzFi65E25C24N7im4
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -429,7 +429,7 @@
     <t xml:space="preserve">Fri Sep 4</t>
   </si>
   <si>
-    <t xml:space="preserve">BRONZE 1910-59 WINNER (64) +25 BRONZE - first win since the Aug 28 Golden Heart, and it carries Bronze past target (152/133). Low Diamond 9-16 (64) +3 D; All-Silver 9-16 (64) +3 PDD. ZERO: 5L Deadball 65-128 (128). Partial day - four events resolved as of 6pm Central, all run numbers exactly +1 on their Sep 3 counterparts.</t>
+    <t xml:space="preserve">BRONZE 1910-59 WINNER (64) +25 BRONZE - first win since the Aug 28 Golden Heart, and it carries Bronze past target (152/133). SILVER ONLY CAP 3rd/4th (64) +10 SILVER/+10 CAP. Low Diamond 9-16 (64) +3 D; All-Silver 9-16 (64) +3 PDD. ZEROS: 5L Deadball 65-128 (128); Low Silver Only 33-64 (64). Partial day - logged 6pm then amended 9pm Central. NOTE: Silver Only Cap came through as run 1250174 where the daily-increment model expects 1250173 for Sep 4 (slot 125 was renamed in the Sep refresh); the game's own Today label and Low Silver Only 1970003 (+1 on Sep 3's 1970002) both put it on Sep 4, so it is filed here.</t>
   </si>
   <si>
     <t xml:space="preserve">The Championship Ladder — PTCS → PTMS → PTWC</t>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUM('Daily Log'!E5:E52)</f>
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>119</v>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">SUM('Daily Log'!J5:J52)</f>
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>161</v>
@@ -2996,7 +2996,7 @@
         <v>25</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F37" s="7" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
         <v>0</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K37" s="7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
PTCS6: Sep 4 to +59 from the results screen, Sep 2 +1; cwhit request list
Read Your Tournaments directly instead of a screenshot and found two Sep 4
results never logged: Gold Slots 9-16 (64, Gld+Cp) +3 G/+3 C and Open Slots
17-32 (64, Op+Cp) +1 O/+1 C. Sep 2 also gains Wednesday Ice to See You
65-128 (256, Dia+TW) +1 D.

Gold 149, Diamond 126, Open 16, Cap 200. Period total 1,171 through day 33.

Adds the cwhit stat-request list: 25 of his missing IDs are still inside the
results window, none of them already in Archive/Completed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RG3WVSzFi65E25C24N7im4
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -417,7 +417,7 @@
     <t xml:space="preserve">Wed Sep 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Wednesday 1950 to Now 17-32 (128, Op+TW) +3 OPEN - counted per the game's own Op tag; note the dump model currently EXCLUDES this event, so it may not show up in the community Open standings. ZEROS: Open Slots 33-64 (64, Op+Cp); Early Gold 65-128 (128). LATE ADDS from the Sep 4 screenshot (+6): Bronze PTCS 3 Replay Slots 1890099 17-32 (64) +1 B/+1 C; All-Diamond 2200173 9-16 (64) +3 PDD; 6L Power Play 2180173 33-64 (128) +1 PDD. LATE ZERO: Wednesday Night of the Living Deadball 1500024 65-128 (128, Op+TW).</t>
+    <t xml:space="preserve">Wednesday 1950 to Now 17-32 (128, Op+TW) +3 OPEN - counted per the game's own Op tag; note the dump model currently EXCLUDES this event, so it may not show up in the community Open standings. ZEROS: Open Slots 33-64 (64, Op+Cp); Early Gold 65-128 (128). LATE ADDS from the Sep 4 screenshot (+6): Bronze PTCS 3 Replay Slots 1890099 17-32 (64) +1 B/+1 C; All-Diamond 2200173 9-16 (64) +3 PDD; 6L Power Play 2180173 33-64 (128) +1 PDD. LATE ZERO: Wednesday Night of the Living Deadball 1500024 65-128 (128, Op+TW). AMENDED from the Sep 4 results screen (+1): Wednesday Ice to See You 1490024 65-128 (256, Dia+TW) +1 D. ADDITIONAL ZEROS: Late Silver 1240173 65-128 (128); Silver &amp; Friends Slots 1900099 33-64 (64). Day complete.</t>
   </si>
   <si>
     <t xml:space="preserve">Thu Sep 3</t>
@@ -429,7 +429,7 @@
     <t xml:space="preserve">Fri Sep 4</t>
   </si>
   <si>
-    <t xml:space="preserve">BRONZE 1910-59 WINNER (64) +25 BRONZE - first win since the Aug 28 Golden Heart, and it carries Bronze past target (152/133). SILVER ONLY CAP 3rd/4th (64) +10 SILVER/+10 CAP. Low Diamond 9-16 (64) +3 D; All-Silver 9-16 (64) +3 PDD. ZEROS: 5L Deadball 65-128 (128); Low Silver Only 33-64 (64). Partial day - logged 6pm then amended 9pm Central. NOTE: Silver Only Cap came through as run 1250174 where the daily-increment model expects 1250173 for Sep 4 (slot 125 was renamed in the Sep refresh); the game's own Today label and Low Silver Only 1970003 (+1 on Sep 3's 1970002) both put it on Sep 4, so it is filed here.</t>
+    <t xml:space="preserve">BRONZE 1910-59 WINNER (64) +25 BRONZE - second win of the period, carries Bronze past target. SILVER ONLY CAP 3rd/4th (64) +10 S/+10 C. Gold Slots 9-16 (64, Gld+Cp) +3 G/+3 C; Low Diamond 9-16 (64) +3 D; Open Slots 17-32 (64, Op+Cp) +1 O/+1 C; All-Silver 9-16 (64) +3 PDD. ZEROS: 5L Deadball 65-128 (128); Low Silver Only 33-64 (64). Read straight off the Your Tournaments screen at 10pm Central, so the tournament side of the day is COMPLETE; PD events are filtered out of that view and may still add. In flight: Silver &amp; Friends Slots 1900101 and Late Silver 1240175 (both eliminated), Diamond &amp; Friends 1920101, Silver Slots 1270175, Diamond Heart 1850158, Saturday Diamond Variety 1590025.</t>
   </si>
   <si>
     <t xml:space="preserve">The Championship Ladder — PTCS → PTMS → PTWC</t>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">SUM('Daily Log'!F5:F52)</f>
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>114</v>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM('Daily Log'!G5:G52)</f>
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>99</v>
@@ -1279,18 +1279,18 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">SUM('Daily Log'!H5:H52)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>120</v>
       </c>
       <c r="D10" s="7" t="n">
         <f aca="false">MAX(0,C10-B10)</f>
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E10" s="7" t="n">
         <f aca="false">ROUND(D10/5,1)</f>
-        <v>21</v>
+        <v>20.8</v>
       </c>
       <c r="F10" s="7" t="n">
         <f aca="false">ROUND(D10/35,1)</f>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="H10" s="9" t="str">
         <f aca="false">IF(B10&gt;=C10,"QUALIFIED","+"&amp;TEXT(D10,"0")&amp;" to go")</f>
-        <v>+105 to go</v>
+        <v>+104 to go</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">SUM('Daily Log'!J5:J52)</f>
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>161</v>
@@ -2920,7 +2920,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>3</v>
@@ -2999,19 +2999,19 @@
         <v>10</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G37" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K37" s="7" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
PTCS 6 days 34-35: Sep 5 amended to 20, Sep 6 (final day) +42 - period closes at 1,252
Sep 5 picks up the six events that were still in flight at the first read
(Late Silver 17-32 +3 S, Saturday Diamond Variety +1 D, Bronze OOTP Era +1 B,
Perfectly Silver +1 PDD). Sep 6: Sunday High Iron Floor / Gold Ceiling 5-8
(128) +10 G/+10 C, Open Slots 5-8 +6 Op/+6 C, Perfecto Morning +6 PDD, Rise
and Shine +3 PDD, All-Silver +1 PDD.

Final: Bronze 154, Silver 170, Gold 159, Diamond 131, Cap 220 - all over the
estimated line; PD Daily 331 (16 short of 347); Open 22, Live 13, PD Weekly
52, Iron 0. Seed JSON, Dashboard DATA and the Tracker Daily Log (rows 38-39)
agree; the DB was imported through Sep 6 already.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121txtos3HpQsWrWtp17C2d
</commit_message>
<xml_diff>
--- a/PTCS6 Tracker.xlsx
+++ b/PTCS6 Tracker.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="200">
   <si>
     <t xml:space="preserve">PTCS 6 — All 10 Categories (Aug 3 – Sep 6)</t>
   </si>
@@ -435,7 +435,13 @@
     <t xml:space="preserve">Sat Sep 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Day 34 of 35, read straight off the Your Tournaments screen with Show: All Tournaments and Drafts. Around the Breakfast Table 2560101 5-8 (64) +6 PDD; Struggling to Sleep - DBL 2240175 9-16 (64) +3 PDD; Don't Forget to Pick up the Kids - Live 2130175 17-32 (64, PD Daily+Live) +1 PDD/+1 LIVE; Bronze 1910-59 1640171 17-32 (64) +1 B; Low Silver Only 1970004 17-32 (64) +1 S; Diamond Heart 1850158 17-32 (64) +1 D. ZEROS: Silver Only Cap 1250175 and Open Slots 1410175 33-64 (64); Midday Perfecto 2530165 33-64 (64); Negro Leagues Slots 1950014 65-128 (128, Op+Cp+TW). UNSCORED: Saturday Shrinkage 2430025 (256, PD WEEKLY) eliminated with no placement. STILL IN FLIGHT and able to add to this day: All-Gold 2120175, Perfectly Bronze 2140175, Just Order Pizza 2170176, Bronze PTCS 3 1890102, Bronze OOTP Era 1820159 (all eliminated, awaiting placement) and All-Diamond 2200176, 6L Power Play 2180176, Late Silver 1240176, Saturday Diamond Variety 1590025, Perfectly Silver 2550165 (still playing).</t>
+    <t xml:space="preserve">Day 34 of 35, read straight off the Your Tournaments screen with Show: All Tournaments and Drafts. Around the Breakfast Table 2560101 5-8 (64) +6 PDD; Struggling to Sleep - DBL 2240175 9-16 (64) +3 PDD; Don't Forget to Pick up the Kids - Live 2130175 17-32 (64, PD Daily+Live) +1 PDD/+1 LIVE; Bronze 1910-59 1640171 17-32 (64) +1 B; Low Silver Only 1970004 17-32 (64) +1 S; Diamond Heart 1850158 17-32 (64) +1 D. ZEROS: Silver Only Cap 1250175 and Open Slots 1410175 33-64 (64); Midday Perfecto 2530165 33-64 (64); Negro Leagues Slots 1950014 65-128 (128, Op+Cp+TW). UNSCORED: Saturday Shrinkage 2430025 (256, PD WEEKLY) eliminated with no placement. STILL IN FLIGHT and able to add to this day: All-Gold 2120175, Perfectly Bronze 2140175, Just Order Pizza 2170176, Bronze PTCS 3 1890102, Bronze OOTP Era 1820159 (all eliminated, awaiting placement) and All-Diamond 2200176, 6L Power Play 2180176, Late Silver 1240176, Saturday Diamond Variety 1590025, Perfectly Silver 2550165 (still playing). RESOLVED from the Sep 6 screen (+6), clearing every event this note listed as in flight: Late Silver 1240176 17-32 (128) +3 S; Saturday Diamond Variety 1590025 33-64 (128, Dia+TW) +1 D; Bronze OOTP Era 1820159 33-64 (128) +1 B; Perfectly Silver 2550165 17-32 (64) +1 PDD. LATE ZEROS: All-Diamond 2200176 33-64 (64); 6L Power Play 2180176 65-128 (128); Just Order Pizza 2170176 33-64 (64); Bronze PTCS 3 Replay Slots 1890102 33-64 (64); Perfectly Bronze 2140175 33-64 (64); All-Gold 2120175 33-64 (64). Day complete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun Sep 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day 35 of 35 — the last qualifying day — read off the Your Tournaments screen. Sunday High Iron Floor and Gold Ceiling 1600025 5-8 (128, Gld+Cp+TW) +10 G/+10 C; Open Slots 1410176 5-8 (64, Op+Cp) +6 OPEN/+6 C; Perfecto Morning 2520165 5-8 (64) +6 PDD; Rise and Shine 2030176 9-16 (64) +3 PDD; All-Silver 2110176 17-32 (64, PD Daily tag only despite the name) +1 PDD. ZEROS: Gold Slots 1320176 33-64 (64, Gld+Cp); Struggling to Sleep - DBL 2240176 33-64 (64). Read across two captures of the Today rows; if anything else finished after the second one, this day is short by that amount.</t>
   </si>
   <si>
     <t xml:space="preserve">The Championship Ladder — PTCS → PTMS → PTWC</t>
@@ -1161,7 +1167,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">SUM('Daily Log'!D5:D52)</f>
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>133</v>
@@ -1192,7 +1198,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUM('Daily Log'!E5:E52)</f>
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>119</v>
@@ -1223,7 +1229,7 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">SUM('Daily Log'!F5:F52)</f>
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>114</v>
@@ -1254,7 +1260,7 @@
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">SUM('Daily Log'!G5:G52)</f>
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>99</v>
@@ -1285,29 +1291,29 @@
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">SUM('Daily Log'!H5:H52)</f>
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>120</v>
       </c>
       <c r="D10" s="7" t="n">
         <f aca="false">MAX(0,C10-B10)</f>
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="E10" s="7" t="n">
         <f aca="false">ROUND(D10/5,1)</f>
-        <v>20.8</v>
+        <v>19.6</v>
       </c>
       <c r="F10" s="7" t="n">
         <f aca="false">ROUND(D10/35,1)</f>
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>20</v>
       </c>
       <c r="H10" s="9" t="str">
         <f aca="false">IF(B10&gt;=C10,"QUALIFIED","+"&amp;TEXT(D10,"0")&amp;" to go")</f>
-        <v>+104 to go</v>
+        <v>+98 to go</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1347,7 +1353,7 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">SUM('Daily Log'!J5:J52)</f>
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>161</v>
@@ -1378,29 +1384,29 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">SUM('Daily Log'!K5:K52)</f>
-        <v>320</v>
+        <v>331</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>347</v>
       </c>
       <c r="D13" s="7" t="n">
         <f aca="false">MAX(0,C13-B13)</f>
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">ROUND(D13/5,1)</f>
-        <v>5.4</v>
+        <v>3.2</v>
       </c>
       <c r="F13" s="7" t="n">
         <f aca="false">ROUND(D13/35,1)</f>
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>26</v>
       </c>
       <c r="H13" s="9" t="str">
         <f aca="false">IF(B13&gt;=C13,"QUALIFIED","+"&amp;TEXT(D13,"0")&amp;" to go")</f>
-        <v>+27 to go</v>
+        <v>+16 to go</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3040,16 +3046,16 @@
         <v>0</v>
       </c>
       <c r="D38" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F38" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H38" s="7" t="n">
         <v>0</v>
@@ -3061,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L38" s="7" t="n">
         <v>0</v>
@@ -3071,19 +3077,45 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="9"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="9"/>
-      <c r="J39" s="9"/>
-      <c r="K39" s="9"/>
-      <c r="L39" s="9"/>
-      <c r="M39" s="9"/>
+      <c r="A39" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="K39" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="L39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="12" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="9"/>
@@ -3309,151 +3341,151 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>142</v>
-      </c>
       <c r="F5" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>300</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>100</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>40</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>20</v>
       </c>
       <c r="D10" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>158</v>
-      </c>
       <c r="F10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="5" t="n">
@@ -3464,7 +3496,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>2</v>
@@ -3472,7 +3504,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>1</v>
@@ -3480,21 +3512,21 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>3</v>
@@ -3505,10 +3537,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C18" s="7" t="n">
         <v>0</v>
@@ -3520,35 +3552,35 @@
         <v>0</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="12" t="s">
         <v>170</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C20" s="7" t="n">
         <v>1</v>
@@ -3560,15 +3592,15 @@
         <v>1</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>20</v>
@@ -3580,15 +3612,15 @@
         <v>20</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C22" s="7" t="n">
         <v>9</v>
@@ -3600,12 +3632,12 @@
         <v>14</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7" t="n">
@@ -3621,52 +3653,52 @@
         <v>35</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3674,17 +3706,17 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3692,17 +3724,17 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3710,7 +3742,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>